<commit_message>
Audit full Day22 requirements and verify current FX
</commit_message>
<xml_diff>
--- a/output/DuongThiHongVien_Day22_model.xlsx
+++ b/output/DuongThiHongVien_Day22_model.xlsx
@@ -3627,7 +3627,7 @@
         <v>191</v>
       </c>
       <c r="B68" s="15">
-        <v>26000</v>
+        <v>26100</v>
       </c>
       <c r="C68" s="3" t="s">
         <v>192</v>
@@ -3642,7 +3642,7 @@
       </c>
       <c r="B69" s="36">
         <f>B66*B68</f>
-        <v>1772.2249999999997</v>
+        <v>1779.0412499999998</v>
       </c>
       <c r="C69" s="3" t="s">
         <v>198</v>

</xml_diff>

<commit_message>
Finalize channel evidence and confirm VLearn submission
</commit_message>
<xml_diff>
--- a/output/DuongThiHongVien_Day22_model.xlsx
+++ b/output/DuongThiHongVien_Day22_model.xlsx
@@ -7880,13 +7880,13 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="95" customHeight="1">
+    <row r="42" ht="163" customHeight="1">
       <c r="A42" s="6" t="s">
         <v>268</v>
       </c>
       <c r="B42" s="45" t="inlineStr">
         <is>
-          <t>Thử self-service nhỏ; đo CAC, dừng nếu chưa có kênh nhập dữ liệu.</t>
+          <t>PLG nhỏ; ICONIQ 2026 p22: SMB CPO $6300, /20%=CAC $31500, 19,78x budget; không phải SME VN. Xem channel-evidence.md.</t>
         </is>
       </c>
       <c r="D42" s="3" t="s">
@@ -9013,13 +9013,13 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="44" customHeight="1">
+    <row r="14" ht="61" customHeight="1">
       <c r="A14" s="6" t="s">
         <v>270</v>
       </c>
       <c r="B14" s="47" t="inlineStr">
         <is>
-          <t>Phỏng vấn buyer + đo ghi chú thủ công.</t>
+          <t>Phỏng vấn buyer; kiểm giả định 20 phút/job x $6/giờ x400=$800/tháng.</t>
         </is>
       </c>
       <c r="C14" s="47" t="inlineStr">
@@ -9033,7 +9033,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="44" customHeight="1">
+    <row r="15" ht="61" customHeight="1">
       <c r="A15" s="6" t="s">
         <v>271</v>
       </c>
@@ -9044,7 +9044,7 @@
       </c>
       <c r="C15" s="47" t="inlineStr">
         <is>
-          <t>Meter jobID; cap 400; đơn giá rõ.</t>
+          <t>Meter jobID; cap400 completed; tối đa3 attempt/job (2 retry); giá$0,40.</t>
         </is>
       </c>
       <c r="D15" s="47" t="inlineStr">

</xml_diff>